<commit_message>
July 2026 sulfide QAQC
</commit_message>
<xml_diff>
--- a/CO2xN/Porewater/1-Sulfide/2026/Datasheets/2026July_LTREB_H2S_Datasheets.xlsx
+++ b/CO2xN/Porewater/1-Sulfide/2026/Datasheets/2026July_LTREB_H2S_Datasheets.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\GlobalChangeEco\Porewater_R scripts &amp; Data\Data\Sulfide Microplate\LTREB\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sinet-my.sharepoint.com/personal/giessnerm_si_edu/Documents/Documents/GitHub/GCREW/GENX/Porewater/1-Sulfide/2026/Datasheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4499AA84-BEDA-4AA7-992D-9710CA7EE46D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{4499AA84-BEDA-4AA7-992D-9710CA7EE46D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C50CD9CF-EF62-43CE-8425-514EA23870C1}"/>
   <bookViews>
-    <workbookView xWindow="30" yWindow="1320" windowWidth="17895" windowHeight="12600" firstSheet="8" activeTab="13" xr2:uid="{23FB6DB2-3641-4E78-A68E-113D11F8B05A}"/>
+    <workbookView xWindow="0" yWindow="1110" windowWidth="16590" windowHeight="11295" firstSheet="9" activeTab="14" xr2:uid="{23FB6DB2-3641-4E78-A68E-113D11F8B05A}"/>
   </bookViews>
   <sheets>
     <sheet name="STD 1" sheetId="1" r:id="rId1"/>
@@ -5848,13 +5848,13 @@
         <v>50</v>
       </c>
       <c r="H18" s="4">
-        <v>250</v>
+        <v>1250</v>
       </c>
       <c r="I18" s="4">
-        <v>250</v>
+        <v>1250</v>
       </c>
       <c r="J18" s="4">
-        <v>250</v>
+        <v>1250</v>
       </c>
       <c r="K18" s="4"/>
       <c r="L18" s="4"/>

</xml_diff>